<commit_message>
docs(README): MobilePaperViewer 항목이 0.77.0의 옛 계약을 말하던 것
breaking 변경(`columns`/`rows`/`fields`/`values` → `children`)이 0.77.0으로 나갔는데
README 220행은 폐기된 계약을 그대로 설명하고 있었다. `_catalog`는 갱신됐지만 README는
빠졌다 — **소비 앱의 LLM이 읽는 건 README다.** 이대로면 없는 prop을 쓴다.

계약·확대 동작·인쇄 스코프 없음까지 새로 적고, 무엇이 왜 깨졌는지를 ⚠ 한 줄로 남긴다
(옛 계약을 쓰던 소비처가 「왜 안 되지」에서 멈추지 않게).

곁들여 발주서 저작 진행분(개수/수량 이름 정합)을 담는다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/kk-baljooseo.xlsx
+++ b/public/kk-baljooseo.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10802"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A05E2FC-2F33-F04A-89CF-600BB0FFE363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FCAB021-B414-864B-8142-FCF1C3D0B23A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13660" yWindow="720" windowWidth="38400" windowHeight="19060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="3280" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="양식" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="72">
   <si>
     <t>{{발행처로고}}</t>
   </si>
@@ -190,6 +190,10 @@
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
   <si>
+    <t>{{부속.개수}}</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
     <t>{{현장주소}}</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
@@ -202,10 +206,6 @@
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">부속 </t>
-    <phoneticPr fontId="8" type="noConversion"/>
-  </si>
-  <si>
     <t>날짜</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
@@ -253,15 +253,7 @@
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
   <si>
-    <t>수량</t>
-    <phoneticPr fontId="8" type="noConversion"/>
-  </si>
-  <si>
     <t>비고</t>
-    <phoneticPr fontId="8" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{부속.수량}}</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
   <si>
@@ -1203,7 +1195,7 @@
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
       <c r="E4" s="32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F4" s="32"/>
       <c r="G4" s="32"/>
@@ -1268,7 +1260,7 @@
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
       <c r="E6" s="31" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F6" s="31"/>
       <c r="G6" s="31"/>
@@ -1369,11 +1361,11 @@
       <c r="M9" s="36"/>
       <c r="N9" s="37"/>
       <c r="O9" s="35" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="P9" s="37"/>
       <c r="Q9" s="35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="R9" s="36"/>
       <c r="S9" s="36"/>
@@ -1406,11 +1398,11 @@
       <c r="M10" s="39"/>
       <c r="N10" s="40"/>
       <c r="O10" s="44" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="P10" s="45"/>
       <c r="Q10" s="41" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="R10" s="42"/>
       <c r="S10" s="42"/>
@@ -1899,7 +1891,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1939,7 +1931,7 @@
         <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -2006,24 +1998,27 @@
     </row>
     <row r="8" spans="1:5" ht="20">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
         <v>11</v>
       </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="20">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
@@ -2032,62 +2027,49 @@
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="20">
       <c r="A11" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="20">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>70</v>
+      </c>
+      <c r="B12" t="s">
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="20">
-      <c r="A13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C13" t="s">
         <v>60</v>
       </c>
-    </row>
+      <c r="E12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="20"/>
     <row r="14" spans="1:5" ht="20"/>
     <row r="15" spans="1:5" ht="20"/>
     <row r="16" spans="1:5" ht="20"/>
@@ -2120,14 +2102,13 @@
     <row r="43" ht="20"/>
     <row r="44" ht="20"/>
     <row r="45" ht="20"/>
-    <row r="46" ht="20"/>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="C2:C77" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C76" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"글자,숫자,금액,날짜,여러 줄,선택,예아니오,이미지"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D77" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D76" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"필수"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>